<commit_message>
fix(website): use __config__ in /try playground samples
The sample template workbooks served by the /try page named their
reserved config sheet `_config`, the pre-0.1.0 format. The current
engine only recognizes the dunder-wrapped `__config__` (ADR-0011),
so the downloaded samples failed to convert and disagreed with the
page's own hint text, which already says `__config__`.

- build-ko-samples.mjs: rename `_config` -> `__config__` (sheet name
  and the subtitle description text).
- build-en-samples.mjs: add a generator for the English samples,
  which were previously hand-committed binaries with no source. It
  mirrors the KO generator and uses `__config__`.
- Regenerate all four static/playground-samples/*.xlsx.

Verified end-to-end: convert() now resolves output_file_pattern from
the config sheet for both EN and KO sample pairs.
</commit_message>
<xml_diff>
--- a/website/static/playground-samples/sample-raw.xlsx
+++ b/website/static/playground-samples/sample-raw.xlsx
@@ -81,23 +81,17 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF217846"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -105,25 +99,19 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF185C37"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,22 +454,23 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -492,7 +481,7 @@
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>18400</v>
       </c>
       <c r="D2" t="s">
@@ -506,7 +495,7 @@
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>7200</v>
       </c>
       <c r="D3" t="s">
@@ -520,7 +509,7 @@
       <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <v>12600</v>
       </c>
       <c r="D4" t="s">
@@ -534,7 +523,7 @@
       <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>9800</v>
       </c>
       <c r="D5" t="s">
@@ -548,7 +537,7 @@
       <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>21300</v>
       </c>
       <c r="D6" t="s">

</xml_diff>

<commit_message>
fix(website): use __config__ in /try playground samples (#60)
Bring user-facing artifacts to the post-0.1.0 reserved-sheet naming (ADR-0011).

- /try playground samples: _config -> __config__ (EN/KO generators + 4 regenerated xlsx; new build-en-samples.mjs).
- conformance docs + src/types.ts ConvertOptions JSDoc + i18n (ja/zh-CN/zh-TW/es): _inputs -> __inputs__.

Verified: convert() resolves output_file_pattern from __config__ for both sample pairs; full CI green.
</commit_message>
<xml_diff>
--- a/website/static/playground-samples/sample-raw.xlsx
+++ b/website/static/playground-samples/sample-raw.xlsx
@@ -81,23 +81,17 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF217846"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -105,25 +99,19 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF185C37"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,22 +454,23 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -492,7 +481,7 @@
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>18400</v>
       </c>
       <c r="D2" t="s">
@@ -506,7 +495,7 @@
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>7200</v>
       </c>
       <c r="D3" t="s">
@@ -520,7 +509,7 @@
       <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <v>12600</v>
       </c>
       <c r="D4" t="s">
@@ -534,7 +523,7 @@
       <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>9800</v>
       </c>
       <c r="D5" t="s">
@@ -548,7 +537,7 @@
       <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>21300</v>
       </c>
       <c r="D6" t="s">

</xml_diff>